<commit_message>
fix(inventory): correct AEC control-cable retirement mass
The AEC balance-of-plant retirement inventory sends 800 kg of cable to treatment for its 100 kg control-unit assembly. The existing native control-unit reference assigns 8% nominal finished mass to cables; PEM and SOEC already retire 8 kg. Separate bulk copper and replacement conversion/drive hardware have their own disposal routes.

Change only the existing AEC used-cable purchase from -800 to -8 kg and document its ownership in the supplemental electrolysis workbook. Preserve manufacturing, metal inputs, energy, equipment allocation and signed waste conventions. This removes 792 kg of unsupported waste without asserting a newly measured control-panel design.

Validation: exact no-write workbook import comparison; isolated full-network EF 3.1 solve and change reconciliation. All other imported exchanges and production signs are unchanged. Only the existing workbook is staged.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-electrolysis.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-electrolysis.xlsx
@@ -14846,7 +14846,9 @@
       </c>
       <c r="B403" s="14" t="inlineStr">
         <is>
-          <t>APPROVED ELECTROLYZER AUXILIARY DRIVE REFERENCES, issue98, 2026-10-18. ABB ACS880-01 R6 environmentalclaim RevB20240619:75kW,46.82kgincludingwood10.7%+cardboard1.3%,10yearlife. R3 EPD RevA20241127:18.5kWrepresentative,range5.5-22kWincludes15kW,11.9kgincludingcardboard11.5%+paper1.7%. R1 claim RevB20240617:5.5kWrepresentative,range0.75-5.5kWincludes1.1kW,8.71kgincludingcardboard8.8%+EPP4.1%. Sources https://library.e.abb.com/public/38ade840ed494fa4864fdb705fed986a/Self-Declared_Environmental_Claim_ACS880-01_R6_3AXD10002202569_RevB_EN_20240619.pdf ; https://library.e.abb.com/public/657ba75f918a4bfe9c6d28b90bc926fa/PEP_EPD_ACS880-01_R3_3AXD10002381313_RevA_EN_20241127.pdf ; https://library.e.abb.com/public/8eb29c5519684381bfc61d575364e663/Self-Declared_Environmental_Claim_ACS880-01_R1_3AXD10002202558_RevB_EN_20240617.pdf . Originalcompressorfrequencyconverter300kg(60Al+45Cu+180reinforcingsteel+15elastomer)containednodedicatedswitches/capacitors/controlparts;SOECfivecopies1500kgplus4.9kgwaterpumpdrive. ReplaceonlytheseexplicitdrivevectorsandCuwiredrawing,notcompressors,motors,100kgplantcontrols,mainrectifier93orotherBoP. Motornameplates/pressurestageallocationwerenotrecovered. ChooseEXPLICITengineeringdutyenvelope75kWaggregatecompressormotorcapacity:one75kWdriveinPEM/AEC;five15kWdrivesinSOEC;one1.1kWwaterpumpdriveinSOEC. Thesearecapacity-matchedREFERENCEASSUMPTIONS,notproofoldplantmotorshadtheseratings. For25kgH2/h,1-&gt;30bar,298K,theisothermalminimum~29kW;75kWenvelopegivesheadroombutPEM/AECpressureconditions/actualstageworkdifferandmustbevalidated. Sensitivitytotal30/75/150kW,onevsfivestagesandoriginalmass-basedrecipe;nonewcompressionlossenergyaddedbecauseexistingH2energydemandretained. R3/R1profiletransferredwithinpublishedframepowerrange,notlinearlyscaledby15/18.5or1.1/5.5. R6knownfractionssteel45,Al14.4,Cu7.2,PC5.3,ABS3.7,electronics7.7wt%ofgross46.82;R3steel19.5,Al22.1,PC18.9,ABS5.1,SEBS0.9,electronics15.7;R1steel16.7,Al16.4,Cu3.4,PC22,ABS8.5,electronics15.4. Percentagesapplytogrosspackagedmass,packagingexcludedfrominstalledweightandmodeledonce. EPDother/missingfractionkeptUNRESOLVED,notallocatedtozero-metalplastic;R3smallCucontentlikelywithinother,notclaimedzeroCu. Electronicscategoryisexplicitpartitionassumption:75kW6halfbridgemodules(3IGBTswitching+3usingintegralantiparalleldiodesaspassivebridge),0.75kgmountedPCB,0.65kgfilmDC-linkcaps,0.05kgfan;15kW12TO2471200Vparts(6switches+6bodydiodesforpassiverectification),1kgmountedPCB,0.6kgcaps,0.05kgfan;1.1kW12TO247650Vparts,0.65kgPCB,0.35kgcaps,0.06kgfan. ThisisCONSERVATIVEsyntheticrectifierchoicewithunusedswitchdies,notABBfittedBOM. Mountedsupplierincludesgate/controlICs;doNOTaddTIgate-driverpackagesagain. Reference0.2mF/kWDC-linkat600V and8kHzswitchingisnotvalidatedripple/thermal/EMIdesign. BulkEPDmetalsareassumedoutsideelectronicscategory;partitionuncertaintymustbesensitivitytested,nodoublecompleteEVinverter. OtherresidualelectronicsunmodelledcompositionisnotzeroAu/Ag/Ta. EPD10yearlifevs20yearBoPmeans2expectedmanufacturing/EOLpurchasesperdrive;5-20yearlifesensitivity. Nooperatingelectricityorlifechangeselsewhere. RemoveoldknowncomponentamountsfromexistingaggregateAl/Cu/reinforcingsteel/plasticEOLandaddonekitWEEErouteformatchednewfinishedmass;legacyrounding/otherBoPwastesunvalidated. Packagingtreatedinmanufactureonce,notinstalledWEEE. Fullcomponentmassandassumptionsdocumented,notuniversalindustrialinventory.
+          <t>CONTROL-CABLE RETIREMENT MASS CORRECTION, 2026-10-20. Existing purchased control-unit assembly:100kg, nominal46%steel/32%industrial plastic/14%mounted boards/8%cables; native ecoinvent control-unit documentation, checked in3.12cutoff RER andRoW. Cable inputs expressed partly in metres are NOT summed as kg. These are retained source assembly fractions, not a newly measured control-panel BOM. Existing inventory sources Gerloff2021 DOI10.1016/j.est.2021.102759 and the separately documented replacement power-conversion/drive kits. For one AEC BoP the100kg control assembly contributes8kg nominal finished cables, not800kg. Correct only its aggregate used-cable treatment purchase from-800 to-8kg. PEM/SOEC already use-8kg. The371.7kg separate AEC copper feed already has its separate approximately372kg scrap-Cu route; it is not an extra800kg cable. Replacement converter and motor-drive disposal remains in its dedicated kit and is not added here. Preserve negative waste production and negative treatment purchase, so actual disposal activation stays positive. Manufacturing, metal purchases, operating energy, stack and equipment lifetimes are unchanged. This removes792kg unsupported waste per BoP; it does not qualify the real cable design or all other BoP waste fractions.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+APPROVED ELECTROLYZER AUXILIARY DRIVE REFERENCES, issue98, 2026-10-18. ABB ACS880-01 R6 environmentalclaim RevB20240619:75kW,46.82kgincludingwood10.7%+cardboard1.3%,10yearlife. R3 EPD RevA20241127:18.5kWrepresentative,range5.5-22kWincludes15kW,11.9kgincludingcardboard11.5%+paper1.7%. R1 claim RevB20240617:5.5kWrepresentative,range0.75-5.5kWincludes1.1kW,8.71kgincludingcardboard8.8%+EPP4.1%. Sources https://library.e.abb.com/public/38ade840ed494fa4864fdb705fed986a/Self-Declared_Environmental_Claim_ACS880-01_R6_3AXD10002202569_RevB_EN_20240619.pdf ; https://library.e.abb.com/public/657ba75f918a4bfe9c6d28b90bc926fa/PEP_EPD_ACS880-01_R3_3AXD10002381313_RevA_EN_20241127.pdf ; https://library.e.abb.com/public/8eb29c5519684381bfc61d575364e663/Self-Declared_Environmental_Claim_ACS880-01_R1_3AXD10002202558_RevB_EN_20240617.pdf . Originalcompressorfrequencyconverter300kg(60Al+45Cu+180reinforcingsteel+15elastomer)containednodedicatedswitches/capacitors/controlparts;SOECfivecopies1500kgplus4.9kgwaterpumpdrive. ReplaceonlytheseexplicitdrivevectorsandCuwiredrawing,notcompressors,motors,100kgplantcontrols,mainrectifier93orotherBoP. Motornameplates/pressurestageallocationwerenotrecovered. ChooseEXPLICITengineeringdutyenvelope75kWaggregatecompressormotorcapacity:one75kWdriveinPEM/AEC;five15kWdrivesinSOEC;one1.1kWwaterpumpdriveinSOEC. Thesearecapacity-matchedREFERENCEASSUMPTIONS,notproofoldplantmotorshadtheseratings. For25kgH2/h,1-&gt;30bar,298K,theisothermalminimum~29kW;75kWenvelopegivesheadroombutPEM/AECpressureconditions/actualstageworkdifferandmustbevalidated. Sensitivitytotal30/75/150kW,onevsfivestagesandoriginalmass-basedrecipe;nonewcompressionlossenergyaddedbecauseexistingH2energydemandretained. R3/R1profiletransferredwithinpublishedframepowerrange,notlinearlyscaledby15/18.5or1.1/5.5. R6knownfractionssteel45,Al14.4,Cu7.2,PC5.3,ABS3.7,electronics7.7wt%ofgross46.82;R3steel19.5,Al22.1,PC18.9,ABS5.1,SEBS0.9,electronics15.7;R1steel16.7,Al16.4,Cu3.4,PC22,ABS8.5,electronics15.4. Percentagesapplytogrosspackagedmass,packagingexcludedfrominstalledweightandmodeledonce. EPDother/missingfractionkeptUNRESOLVED,notallocatedtozero-metalplastic;R3smallCucontentlikelywithinother,notclaimedzeroCu. Electronicscategoryisexplicitpartitionassumption:75kW6halfbridgemodules(3IGBTswitching+3usingintegralantiparalleldiodesaspassivebridge),0.75kgmountedPCB,0.65kgfilmDC-linkcaps,0.05kgfan;15kW12TO2471200Vparts(6switches+6bodydiodesforpassiverectification),1kgmountedPCB,0.6kgcaps,0.05kgfan;1.1kW12TO247650Vparts,0.65kgPCB,0.35kgcaps,0.06kgfan. ThisisCONSERVATIVEsyntheticrectifierchoicewithunusedswitchdies,notABBfittedBOM. Mountedsupplierincludesgate/controlICs;doNOTaddTIgate-driverpackagesagain. Reference0.2mF/kWDC-linkat600V and8kHzswitchingisnotvalidatedripple/thermal/EMIdesign. BulkEPDmetalsareassumedoutsideelectronicscategory;partitionuncertaintymustbesensitivitytested,nodoublecompleteEVinverter. OtherresidualelectronicsunmodelledcompositionisnotzeroAu/Ag/Ta. EPD10yearlifevs20yearBoPmeans2expectedmanufacturing/EOLpurchasesperdrive;5-20yearlifesensitivity. Nooperatingelectricityorlifechangeselsewhere. RemoveoldknowncomponentamountsfromexistingaggregateAl/Cu/reinforcingsteel/plasticEOLandaddonekitWEEErouteformatchednewfinishedmass;legacyrounding/otherBoPwastesunvalidated. Packagingtreatedinmanufactureonce,notinstalledWEEE. Fullcomponentmassandassumptionsdocumented,notuniversalindustrialinventory.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
 APPROVED INDUSTRIAL RECTIFIER/TRANSFORMER HARDWARE REFERENCE, issue93, 2026-10-18. ABB2024DCS880PEP,ABBG-00601-V01.01-EN,pp4-10,industrialDCconverters9-5520kWincludingelectrolysis:reference120.63kgincluding6.8kgpackaging,materialcategoriesperTable;187kgH7familyusedasgrosscabinet-scaleanalogue. https://library.e.abb.com/public/41e28362ad194fb1b6172e296a83ee64/PEP_EPD_DCS880_H1_H8_3AXD10002336256_RevA_EN_20241003.pdf . InfineonFF1000UXTR23T2M1MCD18July2025,1017g,2300VSiChalfbridgemodule: https://www.infineon.com/assets/row/public/documents/60/75/infineon-ff1000uxtr23t2m1-materialcontentdatasheet-en.pdf . IEAPVPS2026DOI10.69766/WJTE1771X-transformer-utilityL,2500kVA20/0.4kVmanufacturer-based5681.2kgoiltransformerprofile(Boutros2026/Schneider2016). Theold1tonne(100Al+200Cu+600steel+100elastomer)power-electronicsblockhadnopart-levelrectifierrecipe. ReplaceonlythatblockinPEM/AEC/SOECBoPs,notcompressor/pumpfrequencyconvertersor100kgplantcontrols. Newone1MWreferencecomprises187kgconverterand1.1MVAtransformer,nominalgrossmass2686.728kg;old1000kgmasswasnotindependentlyvalidatedandisNOTpreservedasmeasuredtruth. Thisis an explicitREFERENCE-DESIGNCHANGErequiringoldbulk-versusnewreferenceandtransformer1.05-1.5MVAsensitivity,notproofthatallsitesneedthismass. Converteris a syntheticactivefront-endengineeringvariant,NOTa certifiedABB_DCS880(whichisthyristor-based). Transferonlyitsindustrialcabinetmaterialprofileand187kgfamilymass;use3documentedSiChalfbridgemodules(6switches)at3*1.017kg,a1MW1100VDC/690VACreference. At98%converterefficiencyand0.99powerfactor,ACcurrent=862.4402397079726A,DCcurrent909.09A;1.1MVAexceeds1MW/(.98*.99). Semiconductorvoltage2300Vhasheadroom;Transformerleakageisassumedtoprovideinputreactanceinthedeclaredreference;actualneedforadditionallinechokes/EMIfiltersis anunresolveddesigngap,notclaimedzeroequipment. Actualjunctiontemperature,ripple,DCstackvoltage,controlstabilityandcoolingMUSTbevalidatedforarealdesign. Module is anindustrial/renewablespowerpart,notanEVinverterinventory. Threepartsare a topologyassumption,notsourcedABBfittedcount. Factory2025/26designisananalogueforstaticinventoryyears,notmeasured2020installedtechnology. MCDknownretainedfractions={'Cu': 0.68, 'Sn': 0.016, 'SiC': 0.001, 'Si3N4': 0.009, 'Ni': 0.001, 'Sb': 0.001, 'Ag': 0.001, 'silicone': 0.084, 'PA': 0.089, 'glass': 0.046, 'orgP': 0.015, 'steel': 0.05, 'carbon': 0.001, 'PbO': 1.8e-05};sum=0.9940180000000001,remainder=0.005981999999999932unquantifiedtrace/rounding/otheradditives. Gold,Co,Y,Mg,Zn,CrtracesmarkedXareUNQUANTIFIED,notzero. Usefullknownmaterialfeedonce,100%finalassemblyreference;nativefeedproductionyieldremains. SiCpowderandstoichiometricSi3N4arefeed-gradeproxies;semiconductorwafer/epitaxy/dieyieldandpurificationenergyareunresolved,notrepresentedbyanextraall-siliconICTchip. Si3N4=3Si+2N2with3MJ/kgheat+1kWh/kgengineeringmanufacture;PbO=Pb+Owith3MJ/kgheat. Convertergrosscategoryledger={'ABS': 8.12501282614425, 'GFplastic': 7.530499692523939, 'PA': 1.3871973117807257, 'steel': 53.308010981287886, 'Al': 42.80494562066239, 'Cu': 39.832379952560835, 'electronics': 29.131143547395236, 'other': 2.5762235790213475}. EPDpercentagesandpackagingareincomplete/rounded:retainknownabsoluteamountson120.63kg/113.83kgproductbasis;doNOTrenormalizecategoriesorapplypackagingasinstalledproduct. Knownbulkmetals/plasticsplusmoduleingredientsaremodeled. Electronicscategorypartition:3.051kgcompletepowermodules,8kgmountedgate/protectionPCBs,14kgfilmDC-linkcapacitors,1kgcoolingblower,remaining3.080143547395238kgUNRESOLVED. ThesePCB/capacitor/fanmassallocationsareengineeringassumptionswith50-150%sensitivity,notmanufacturerBOM.14kgcapbankreference5mFat1100Vstores3.025kJ;actualESR/ripple/hold-up/temperaturequalificationunknown. Fanusesgenericperkgcoolingfanmaterialproxy,notverifiedindustrialairflow. KeepunknownEPDother/missingmass=4.880810067644745kgplusunknownmodulefractionexplicit;doNOTassigntoallPCB,gold-freepolymeroranyinventedmetal. GFthermoplasticuses70%PA/30%glassfibreengineeringcomposition;polymergrades/flameretardantsunknown. Transformeris .44 ofsource2500kVAprofileatfixedmaterialperVAasexplicitlinearcapacityassumption,notnonlinearsizinglaw. ExistingLVgridsupplyretained:dedicatedtransformerassumedon-site400/690Visolation/voltageadaptation;20/0.4kVsourcecoil/insulationgeometryisMATERIALSCALEPROXY,notexactturnsratiodesign. Nativepublic-griddistributionhardwareanddedicatedplanttransformerareseparatefunctions. NominalsourceGOES2153kgusesexplicit3wt%Si+97%unalloyedsteelreference;thermal/rollingprocessesretainedandscaled. Sourcepressboard36.96isMASSkg,not36.96m3;convertathardboard1000kg/m3reference(800-1300sensitivity). Listedsourceingredients5670kgversusdeclared5681.2kg:11.2kgremainunresolved,notfilledwithmetal. Thislocaltransformerreferencecorrectsunit/compositiononlywithinthisnewprovider;existingPVworkbookunchanged. ManufacturingONLYinnewhardwarehelpers;existingplantassemblyelectricityretained,noextraoperatinglossenergyorstandby. Lifetime20yearBoPallocationandstacklifeunchanged. UpdateexistingBoPEOLvectorsbyremovingoldpowerblock600kgsteel/100kgAl/200kgCu/100kgplastic,andaddonecompletepower-conversiontreatment. NewEOLroutesknowntransformermetals,cabinetbulkmetals,oil,cellulose,epoxy/rubber/paint,andremainingconvertermassonce;unresolvedtransformermassandmixedminor-metalfatesremaincoveragegaps. No EPDmoduleDcredits,providerrecyclingsharechanges,native/runtime/YAMLmutations.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
@@ -15154,7 +15156,7 @@
         <v>219</v>
       </c>
       <c r="B415" s="11">
-        <v>-800</v>
+        <v>-8.0</v>
       </c>
       <c r="C415" s="11" t="s">
         <v>17</v>
@@ -15167,6 +15169,11 @@
       </c>
       <c r="G415" s="11" t="s">
         <v>220</v>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>CONTROL-CABLE RETIREMENT MASS CORRECTION, 2026-10-20. Existing purchased control-unit assembly:100kg, nominal46%steel/32%industrial plastic/14%mounted boards/8%cables; native ecoinvent control-unit documentation, checked in3.12cutoff RER andRoW. Cable inputs expressed partly in metres are NOT summed as kg. These are retained source assembly fractions, not a newly measured control-panel BOM. Existing inventory sources Gerloff2021 DOI10.1016/j.est.2021.102759 and the separately documented replacement power-conversion/drive kits. For one AEC BoP the100kg control assembly contributes8kg nominal finished cables, not800kg. Correct only its aggregate used-cable treatment purchase from-800 to-8kg. PEM/SOEC already use-8kg. The371.7kg separate AEC copper feed already has its separate approximately372kg scrap-Cu route; it is not an extra800kg cable. Replacement converter and motor-drive disposal remains in its dedicated kit and is not added here. Preserve negative waste production and negative treatment purchase, so actual disposal activation stays positive. Manufacturing, metal purchases, operating energy, stack and equipment lifetimes are unchanged. This removes792kg unsupported waste per BoP; it does not qualify the real cable design or all other BoP waste fractions.</t>
+        </is>
       </c>
       <c r="J415"/>
       <c r="K415" s="19"/>

</xml_diff>

<commit_message>
fix(inventory): reconcile SOEC balance-of-plant steel retirement
The nominal SOEC material ledger buys 19,969 kg ordinary/stainless steel, 46 kg control housing steel and 12,633.6 kg reinforcement. Its disposal rows instead send 20,421 kg to scrap steel and 12,227 kg to reinforcement sorting, misclassifying about 406 kg and retaining 0.6 kg rounding.

Set the two existing waste purchases to -20,015 and -12,633.6 kg. Count metal feeds once, excluding forming-service kilograms. Preserve the separate cast-iron route and dedicated transformer/converter/replacement-drive treatment kit. No manufacture, metal feed, lifetime, operating-energy, supplier or recycling-credit changes. The source-version steel name is retained for existing version migration.

Validation: exact no-write import comparison and isolated full-network EF 3.1 solve/change reconciliation. Workbook comments document the source sums and nominal-design limitation. Only the existing workbook is staged.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-electrolysis.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-electrolysis.xlsx
@@ -19819,7 +19819,9 @@
       </c>
       <c r="B577" s="14" t="inlineStr">
         <is>
-          <t>APPROVED ELECTROLYZER AUXILIARY DRIVE REFERENCES, issue98, 2026-10-18. ABB ACS880-01 R6 environmentalclaim RevB20240619:75kW,46.82kgincludingwood10.7%+cardboard1.3%,10yearlife. R3 EPD RevA20241127:18.5kWrepresentative,range5.5-22kWincludes15kW,11.9kgincludingcardboard11.5%+paper1.7%. R1 claim RevB20240617:5.5kWrepresentative,range0.75-5.5kWincludes1.1kW,8.71kgincludingcardboard8.8%+EPP4.1%. Sources https://library.e.abb.com/public/38ade840ed494fa4864fdb705fed986a/Self-Declared_Environmental_Claim_ACS880-01_R6_3AXD10002202569_RevB_EN_20240619.pdf ; https://library.e.abb.com/public/657ba75f918a4bfe9c6d28b90bc926fa/PEP_EPD_ACS880-01_R3_3AXD10002381313_RevA_EN_20241127.pdf ; https://library.e.abb.com/public/8eb29c5519684381bfc61d575364e663/Self-Declared_Environmental_Claim_ACS880-01_R1_3AXD10002202558_RevB_EN_20240617.pdf . Originalcompressorfrequencyconverter300kg(60Al+45Cu+180reinforcingsteel+15elastomer)containednodedicatedswitches/capacitors/controlparts;SOECfivecopies1500kgplus4.9kgwaterpumpdrive. ReplaceonlytheseexplicitdrivevectorsandCuwiredrawing,notcompressors,motors,100kgplantcontrols,mainrectifier93orotherBoP. Motornameplates/pressurestageallocationwerenotrecovered. ChooseEXPLICITengineeringdutyenvelope75kWaggregatecompressormotorcapacity:one75kWdriveinPEM/AEC;five15kWdrivesinSOEC;one1.1kWwaterpumpdriveinSOEC. Thesearecapacity-matchedREFERENCEASSUMPTIONS,notproofoldplantmotorshadtheseratings. For25kgH2/h,1-&gt;30bar,298K,theisothermalminimum~29kW;75kWenvelopegivesheadroombutPEM/AECpressureconditions/actualstageworkdifferandmustbevalidated. Sensitivitytotal30/75/150kW,onevsfivestagesandoriginalmass-basedrecipe;nonewcompressionlossenergyaddedbecauseexistingH2energydemandretained. R3/R1profiletransferredwithinpublishedframepowerrange,notlinearlyscaledby15/18.5or1.1/5.5. R6knownfractionssteel45,Al14.4,Cu7.2,PC5.3,ABS3.7,electronics7.7wt%ofgross46.82;R3steel19.5,Al22.1,PC18.9,ABS5.1,SEBS0.9,electronics15.7;R1steel16.7,Al16.4,Cu3.4,PC22,ABS8.5,electronics15.4. Percentagesapplytogrosspackagedmass,packagingexcludedfrominstalledweightandmodeledonce. EPDother/missingfractionkeptUNRESOLVED,notallocatedtozero-metalplastic;R3smallCucontentlikelywithinother,notclaimedzeroCu. Electronicscategoryisexplicitpartitionassumption:75kW6halfbridgemodules(3IGBTswitching+3usingintegralantiparalleldiodesaspassivebridge),0.75kgmountedPCB,0.65kgfilmDC-linkcaps,0.05kgfan;15kW12TO2471200Vparts(6switches+6bodydiodesforpassiverectification),1kgmountedPCB,0.6kgcaps,0.05kgfan;1.1kW12TO247650Vparts,0.65kgPCB,0.35kgcaps,0.06kgfan. ThisisCONSERVATIVEsyntheticrectifierchoicewithunusedswitchdies,notABBfittedBOM. Mountedsupplierincludesgate/controlICs;doNOTaddTIgate-driverpackagesagain. Reference0.2mF/kWDC-linkat600V and8kHzswitchingisnotvalidatedripple/thermal/EMIdesign. BulkEPDmetalsareassumedoutsideelectronicscategory;partitionuncertaintymustbesensitivitytested,nodoublecompleteEVinverter. OtherresidualelectronicsunmodelledcompositionisnotzeroAu/Ag/Ta. EPD10yearlifevs20yearBoPmeans2expectedmanufacturing/EOLpurchasesperdrive;5-20yearlifesensitivity. Nooperatingelectricityorlifechangeselsewhere. RemoveoldknowncomponentamountsfromexistingaggregateAl/Cu/reinforcingsteel/plasticEOLandaddonekitWEEErouteformatchednewfinishedmass;legacyrounding/otherBoPwastesunvalidated. Packagingtreatedinmanufactureonce,notinstalledWEEE. Fullcomponentmassandassumptionsdocumented,notuniversalindustrialinventory.
+          <t>SOEC BoP STEEL RETIREMENT RECONCILIATION, 2026-10-20. Existing purchased control-unit assembly:100kg, nominal46%steel/32%industrial plastic/14%mounted boards/8%cables; native ecoinvent control-unit documentation, checked in3.12cutoff RER andRoW. Cable inputs expressed partly in metres are NOT summed as kg. These are retained source assembly fractions, not a newly measured control-panel BOM. Existing inventory sources Gerloff2021 DOI10.1016/j.est.2021.102759 and the separately documented replacement power-conversion/drive kits. Read retained material purchases, not the separate forming-service kg:ordinary/stainless steel16215.4+1503.6+2250=19969kg, plus46kg control housing gives20015kg to existing scrap-steel route. Reinforcing steel6500+5000+8.5+452.1+399+7+267=12633.6kg to its existing sorting route. Previous20421kg scrap steel and12227kg reinforcement misplaced approximately406kg between routes and retained0.6kg source rounding. Correct these two amounts only. Cast iron3000kg has its separate route. All new transformer, converter and replacement-drive metals remain handled by their separate treatment kit: do not add them to these totals again. Manufacturing, metal feeds, operating energy, lifetimes, waste signs and supplier identities are unchanged. This reconciles the existing nominal material ledger, not actual plant grades or recycling recovery fractions; no avoided-production credit.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+APPROVED ELECTROLYZER AUXILIARY DRIVE REFERENCES, issue98, 2026-10-18. ABB ACS880-01 R6 environmentalclaim RevB20240619:75kW,46.82kgincludingwood10.7%+cardboard1.3%,10yearlife. R3 EPD RevA20241127:18.5kWrepresentative,range5.5-22kWincludes15kW,11.9kgincludingcardboard11.5%+paper1.7%. R1 claim RevB20240617:5.5kWrepresentative,range0.75-5.5kWincludes1.1kW,8.71kgincludingcardboard8.8%+EPP4.1%. Sources https://library.e.abb.com/public/38ade840ed494fa4864fdb705fed986a/Self-Declared_Environmental_Claim_ACS880-01_R6_3AXD10002202569_RevB_EN_20240619.pdf ; https://library.e.abb.com/public/657ba75f918a4bfe9c6d28b90bc926fa/PEP_EPD_ACS880-01_R3_3AXD10002381313_RevA_EN_20241127.pdf ; https://library.e.abb.com/public/8eb29c5519684381bfc61d575364e663/Self-Declared_Environmental_Claim_ACS880-01_R1_3AXD10002202558_RevB_EN_20240617.pdf . Originalcompressorfrequencyconverter300kg(60Al+45Cu+180reinforcingsteel+15elastomer)containednodedicatedswitches/capacitors/controlparts;SOECfivecopies1500kgplus4.9kgwaterpumpdrive. ReplaceonlytheseexplicitdrivevectorsandCuwiredrawing,notcompressors,motors,100kgplantcontrols,mainrectifier93orotherBoP. Motornameplates/pressurestageallocationwerenotrecovered. ChooseEXPLICITengineeringdutyenvelope75kWaggregatecompressormotorcapacity:one75kWdriveinPEM/AEC;five15kWdrivesinSOEC;one1.1kWwaterpumpdriveinSOEC. Thesearecapacity-matchedREFERENCEASSUMPTIONS,notproofoldplantmotorshadtheseratings. For25kgH2/h,1-&gt;30bar,298K,theisothermalminimum~29kW;75kWenvelopegivesheadroombutPEM/AECpressureconditions/actualstageworkdifferandmustbevalidated. Sensitivitytotal30/75/150kW,onevsfivestagesandoriginalmass-basedrecipe;nonewcompressionlossenergyaddedbecauseexistingH2energydemandretained. R3/R1profiletransferredwithinpublishedframepowerrange,notlinearlyscaledby15/18.5or1.1/5.5. R6knownfractionssteel45,Al14.4,Cu7.2,PC5.3,ABS3.7,electronics7.7wt%ofgross46.82;R3steel19.5,Al22.1,PC18.9,ABS5.1,SEBS0.9,electronics15.7;R1steel16.7,Al16.4,Cu3.4,PC22,ABS8.5,electronics15.4. Percentagesapplytogrosspackagedmass,packagingexcludedfrominstalledweightandmodeledonce. EPDother/missingfractionkeptUNRESOLVED,notallocatedtozero-metalplastic;R3smallCucontentlikelywithinother,notclaimedzeroCu. Electronicscategoryisexplicitpartitionassumption:75kW6halfbridgemodules(3IGBTswitching+3usingintegralantiparalleldiodesaspassivebridge),0.75kgmountedPCB,0.65kgfilmDC-linkcaps,0.05kgfan;15kW12TO2471200Vparts(6switches+6bodydiodesforpassiverectification),1kgmountedPCB,0.6kgcaps,0.05kgfan;1.1kW12TO247650Vparts,0.65kgPCB,0.35kgcaps,0.06kgfan. ThisisCONSERVATIVEsyntheticrectifierchoicewithunusedswitchdies,notABBfittedBOM. Mountedsupplierincludesgate/controlICs;doNOTaddTIgate-driverpackagesagain. Reference0.2mF/kWDC-linkat600V and8kHzswitchingisnotvalidatedripple/thermal/EMIdesign. BulkEPDmetalsareassumedoutsideelectronicscategory;partitionuncertaintymustbesensitivitytested,nodoublecompleteEVinverter. OtherresidualelectronicsunmodelledcompositionisnotzeroAu/Ag/Ta. EPD10yearlifevs20yearBoPmeans2expectedmanufacturing/EOLpurchasesperdrive;5-20yearlifesensitivity. Nooperatingelectricityorlifechangeselsewhere. RemoveoldknowncomponentamountsfromexistingaggregateAl/Cu/reinforcingsteel/plasticEOLandaddonekitWEEErouteformatchednewfinishedmass;legacyrounding/otherBoPwastesunvalidated. Packagingtreatedinmanufactureonce,notinstalledWEEE. Fullcomponentmassandassumptionsdocumented,notuniversalindustrialinventory.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
 APPROVED INDUSTRIAL RECTIFIER/TRANSFORMER HARDWARE REFERENCE, issue93, 2026-10-18. ABB2024DCS880PEP,ABBG-00601-V01.01-EN,pp4-10,industrialDCconverters9-5520kWincludingelectrolysis:reference120.63kgincluding6.8kgpackaging,materialcategoriesperTable;187kgH7familyusedasgrosscabinet-scaleanalogue. https://library.e.abb.com/public/41e28362ad194fb1b6172e296a83ee64/PEP_EPD_DCS880_H1_H8_3AXD10002336256_RevA_EN_20241003.pdf . InfineonFF1000UXTR23T2M1MCD18July2025,1017g,2300VSiChalfbridgemodule: https://www.infineon.com/assets/row/public/documents/60/75/infineon-ff1000uxtr23t2m1-materialcontentdatasheet-en.pdf . IEAPVPS2026DOI10.69766/WJTE1771X-transformer-utilityL,2500kVA20/0.4kVmanufacturer-based5681.2kgoiltransformerprofile(Boutros2026/Schneider2016). Theold1tonne(100Al+200Cu+600steel+100elastomer)power-electronicsblockhadnopart-levelrectifierrecipe. ReplaceonlythatblockinPEM/AEC/SOECBoPs,notcompressor/pumpfrequencyconvertersor100kgplantcontrols. Newone1MWreferencecomprises187kgconverterand1.1MVAtransformer,nominalgrossmass2686.728kg;old1000kgmasswasnotindependentlyvalidatedandisNOTpreservedasmeasuredtruth. Thisis an explicitREFERENCE-DESIGNCHANGErequiringoldbulk-versusnewreferenceandtransformer1.05-1.5MVAsensitivity,notproofthatallsitesneedthismass. Converteris a syntheticactivefront-endengineeringvariant,NOTa certifiedABB_DCS880(whichisthyristor-based). Transferonlyitsindustrialcabinetmaterialprofileand187kgfamilymass;use3documentedSiChalfbridgemodules(6switches)at3*1.017kg,a1MW1100VDC/690VACreference. At98%converterefficiencyand0.99powerfactor,ACcurrent=862.4402397079726A,DCcurrent909.09A;1.1MVAexceeds1MW/(.98*.99). Semiconductorvoltage2300Vhasheadroom;Transformerleakageisassumedtoprovideinputreactanceinthedeclaredreference;actualneedforadditionallinechokes/EMIfiltersis anunresolveddesigngap,notclaimedzeroequipment. Actualjunctiontemperature,ripple,DCstackvoltage,controlstabilityandcoolingMUSTbevalidatedforarealdesign. Module is anindustrial/renewablespowerpart,notanEVinverterinventory. Threepartsare a topologyassumption,notsourcedABBfittedcount. Factory2025/26designisananalogueforstaticinventoryyears,notmeasured2020installedtechnology. MCDknownretainedfractions={'Cu': 0.68, 'Sn': 0.016, 'SiC': 0.001, 'Si3N4': 0.009, 'Ni': 0.001, 'Sb': 0.001, 'Ag': 0.001, 'silicone': 0.084, 'PA': 0.089, 'glass': 0.046, 'orgP': 0.015, 'steel': 0.05, 'carbon': 0.001, 'PbO': 1.8e-05};sum=0.9940180000000001,remainder=0.005981999999999932unquantifiedtrace/rounding/otheradditives. Gold,Co,Y,Mg,Zn,CrtracesmarkedXareUNQUANTIFIED,notzero. Usefullknownmaterialfeedonce,100%finalassemblyreference;nativefeedproductionyieldremains. SiCpowderandstoichiometricSi3N4arefeed-gradeproxies;semiconductorwafer/epitaxy/dieyieldandpurificationenergyareunresolved,notrepresentedbyanextraall-siliconICTchip. Si3N4=3Si+2N2with3MJ/kgheat+1kWh/kgengineeringmanufacture;PbO=Pb+Owith3MJ/kgheat. Convertergrosscategoryledger={'ABS': 8.12501282614425, 'GFplastic': 7.530499692523939, 'PA': 1.3871973117807257, 'steel': 53.308010981287886, 'Al': 42.80494562066239, 'Cu': 39.832379952560835, 'electronics': 29.131143547395236, 'other': 2.5762235790213475}. EPDpercentagesandpackagingareincomplete/rounded:retainknownabsoluteamountson120.63kg/113.83kgproductbasis;doNOTrenormalizecategoriesorapplypackagingasinstalledproduct. Knownbulkmetals/plasticsplusmoduleingredientsaremodeled. Electronicscategorypartition:3.051kgcompletepowermodules,8kgmountedgate/protectionPCBs,14kgfilmDC-linkcapacitors,1kgcoolingblower,remaining3.080143547395238kgUNRESOLVED. ThesePCB/capacitor/fanmassallocationsareengineeringassumptionswith50-150%sensitivity,notmanufacturerBOM.14kgcapbankreference5mFat1100Vstores3.025kJ;actualESR/ripple/hold-up/temperaturequalificationunknown. Fanusesgenericperkgcoolingfanmaterialproxy,notverifiedindustrialairflow. KeepunknownEPDother/missingmass=4.880810067644745kgplusunknownmodulefractionexplicit;doNOTassigntoallPCB,gold-freepolymeroranyinventedmetal. GFthermoplasticuses70%PA/30%glassfibreengineeringcomposition;polymergrades/flameretardantsunknown. Transformeris .44 ofsource2500kVAprofileatfixedmaterialperVAasexplicitlinearcapacityassumption,notnonlinearsizinglaw. ExistingLVgridsupplyretained:dedicatedtransformerassumedon-site400/690Visolation/voltageadaptation;20/0.4kVsourcecoil/insulationgeometryisMATERIALSCALEPROXY,notexactturnsratiodesign. Nativepublic-griddistributionhardwareanddedicatedplanttransformerareseparatefunctions. NominalsourceGOES2153kgusesexplicit3wt%Si+97%unalloyedsteelreference;thermal/rollingprocessesretainedandscaled. Sourcepressboard36.96isMASSkg,not36.96m3;convertathardboard1000kg/m3reference(800-1300sensitivity). Listedsourceingredients5670kgversusdeclared5681.2kg:11.2kgremainunresolved,notfilledwithmetal. Thislocaltransformerreferencecorrectsunit/compositiononlywithinthisnewprovider;existingPVworkbookunchanged. ManufacturingONLYinnewhardwarehelpers;existingplantassemblyelectricityretained,noextraoperatinglossenergyorstandby. Lifetime20yearBoPallocationandstacklifeunchanged. UpdateexistingBoPEOLvectorsbyremovingoldpowerblock600kgsteel/100kgAl/200kgCu/100kgplastic,andaddonecompletepower-conversiontreatment. NewEOLroutesknowntransformermetals,cabinetbulkmetals,oil,cellulose,epoxy/rubber/paint,andremainingconvertermassonce;unresolvedtransformermassandmixedminor-metalfatesremaincoveragegaps. No EPDmoduleDcredits,providerrecyclingsharechanges,native/runtime/YAMLmutations.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
@@ -19972,7 +19974,7 @@
         <v>204</v>
       </c>
       <c r="B584" s="11">
-        <v>-20421</v>
+        <v>-20015.0</v>
       </c>
       <c r="C584" s="11" t="s">
         <v>37</v>
@@ -19985,6 +19987,11 @@
       </c>
       <c r="G584" s="11" t="s">
         <v>205</v>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>SOEC BoP STEEL RETIREMENT RECONCILIATION, 2026-10-20. Existing purchased control-unit assembly:100kg, nominal46%steel/32%industrial plastic/14%mounted boards/8%cables; native ecoinvent control-unit documentation, checked in3.12cutoff RER andRoW. Cable inputs expressed partly in metres are NOT summed as kg. These are retained source assembly fractions, not a newly measured control-panel BOM. Existing inventory sources Gerloff2021 DOI10.1016/j.est.2021.102759 and the separately documented replacement power-conversion/drive kits. Read retained material purchases, not the separate forming-service kg:ordinary/stainless steel16215.4+1503.6+2250=19969kg, plus46kg control housing gives20015kg to existing scrap-steel route. Reinforcing steel6500+5000+8.5+452.1+399+7+267=12633.6kg to its existing sorting route. Previous20421kg scrap steel and12227kg reinforcement misplaced approximately406kg between routes and retained0.6kg source rounding. Correct these two amounts only. Cast iron3000kg has its separate route. All new transformer, converter and replacement-drive metals remain handled by their separate treatment kit: do not add them to these totals again. Manufacturing, metal feeds, operating energy, lifetimes, waste signs and supplier identities are unchanged. This reconciles the existing nominal material ledger, not actual plant grades or recycling recovery fractions; no avoided-production credit.</t>
+        </is>
       </c>
       <c r="J584"/>
       <c r="K584" s="19"/>
@@ -20001,7 +20008,7 @@
         <v>449</v>
       </c>
       <c r="B585" s="11">
-        <v>-12227</v>
+        <v>-12633.6</v>
       </c>
       <c r="C585" s="11" t="s">
         <v>217</v>
@@ -20017,7 +20024,7 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>APPROVED ELECTROLYZER AUXILIARY DRIVE REFERENCES, issue98, 2026-10-18. ABB ACS880-01 R6 environmentalclaim RevB20240619:75kW,46.82kgincludingwood10.7%+cardboard1.3%,10yearlife. R3 EPD RevA20241127:18.5kWrepresentative,range5.5-22kWincludes15kW,11.9kgincludingcardboard11.5%+paper1.7%. R1 claim RevB20240617:5.5kWrepresentative,range0.75-5.5kWincludes1.1kW,8.71kgincludingcardboard8.8%+EPP4.1%. Sources https://library.e.abb.com/public/38ade840ed494fa4864fdb705fed986a/Self-Declared_Environmental_Claim_ACS880-01_R6_3AXD10002202569_RevB_EN_20240619.pdf ; https://library.e.abb.com/public/657ba75f918a4bfe9c6d28b90bc926fa/PEP_EPD_ACS880-01_R3_3AXD10002381313_RevA_EN_20241127.pdf ; https://library.e.abb.com/public/8eb29c5519684381bfc61d575364e663/Self-Declared_Environmental_Claim_ACS880-01_R1_3AXD10002202558_RevB_EN_20240617.pdf . Originalcompressorfrequencyconverter300kg(60Al+45Cu+180reinforcingsteel+15elastomer)containednodedicatedswitches/capacitors/controlparts;SOECfivecopies1500kgplus4.9kgwaterpumpdrive. ReplaceonlytheseexplicitdrivevectorsandCuwiredrawing,notcompressors,motors,100kgplantcontrols,mainrectifier93orotherBoP. Motornameplates/pressurestageallocationwerenotrecovered. ChooseEXPLICITengineeringdutyenvelope75kWaggregatecompressormotorcapacity:one75kWdriveinPEM/AEC;five15kWdrivesinSOEC;one1.1kWwaterpumpdriveinSOEC. Thesearecapacity-matchedREFERENCEASSUMPTIONS,notproofoldplantmotorshadtheseratings. For25kgH2/h,1-&gt;30bar,298K,theisothermalminimum~29kW;75kWenvelopegivesheadroombutPEM/AECpressureconditions/actualstageworkdifferandmustbevalidated. Sensitivitytotal30/75/150kW,onevsfivestagesandoriginalmass-basedrecipe;nonewcompressionlossenergyaddedbecauseexistingH2energydemandretained. R3/R1profiletransferredwithinpublishedframepowerrange,notlinearlyscaledby15/18.5or1.1/5.5. R6knownfractionssteel45,Al14.4,Cu7.2,PC5.3,ABS3.7,electronics7.7wt%ofgross46.82;R3steel19.5,Al22.1,PC18.9,ABS5.1,SEBS0.9,electronics15.7;R1steel16.7,Al16.4,Cu3.4,PC22,ABS8.5,electronics15.4. Percentagesapplytogrosspackagedmass,packagingexcludedfrominstalledweightandmodeledonce. EPDother/missingfractionkeptUNRESOLVED,notallocatedtozero-metalplastic;R3smallCucontentlikelywithinother,notclaimedzeroCu. Electronicscategoryisexplicitpartitionassumption:75kW6halfbridgemodules(3IGBTswitching+3usingintegralantiparalleldiodesaspassivebridge),0.75kgmountedPCB,0.65kgfilmDC-linkcaps,0.05kgfan;15kW12TO2471200Vparts(6switches+6bodydiodesforpassiverectification),1kgmountedPCB,0.6kgcaps,0.05kgfan;1.1kW12TO247650Vparts,0.65kgPCB,0.35kgcaps,0.06kgfan. ThisisCONSERVATIVEsyntheticrectifierchoicewithunusedswitchdies,notABBfittedBOM. Mountedsupplierincludesgate/controlICs;doNOTaddTIgate-driverpackagesagain. Reference0.2mF/kWDC-linkat600V and8kHzswitchingisnotvalidatedripple/thermal/EMIdesign. BulkEPDmetalsareassumedoutsideelectronicscategory;partitionuncertaintymustbesensitivitytested,nodoublecompleteEVinverter. OtherresidualelectronicsunmodelledcompositionisnotzeroAu/Ag/Ta. EPD10yearlifevs20yearBoPmeans2expectedmanufacturing/EOLpurchasesperdrive;5-20yearlifesensitivity. Nooperatingelectricityorlifechangeselsewhere. RemoveoldknowncomponentamountsfromexistingaggregateAl/Cu/reinforcingsteel/plasticEOLandaddonekitWEEErouteformatchednewfinishedmass;legacyrounding/otherBoPwastesunvalidated. Packagingtreatedinmanufactureonce,notinstalledWEEE. Fullcomponentmassandassumptionsdocumented,notuniversalindustrialinventory.</t>
+          <t>SOEC BoP STEEL RETIREMENT RECONCILIATION, 2026-10-20. Existing purchased control-unit assembly:100kg, nominal46%steel/32%industrial plastic/14%mounted boards/8%cables; native ecoinvent control-unit documentation, checked in3.12cutoff RER andRoW. Cable inputs expressed partly in metres are NOT summed as kg. These are retained source assembly fractions, not a newly measured control-panel BOM. Existing inventory sources Gerloff2021 DOI10.1016/j.est.2021.102759 and the separately documented replacement power-conversion/drive kits. Read retained material purchases, not the separate forming-service kg:ordinary/stainless steel16215.4+1503.6+2250=19969kg, plus46kg control housing gives20015kg to existing scrap-steel route. Reinforcing steel6500+5000+8.5+452.1+399+7+267=12633.6kg to its existing sorting route. Previous20421kg scrap steel and12227kg reinforcement misplaced approximately406kg between routes and retained0.6kg source rounding. Correct these two amounts only. Cast iron3000kg has its separate route. All new transformer, converter and replacement-drive metals remain handled by their separate treatment kit: do not add them to these totals again. Manufacturing, metal feeds, operating energy, lifetimes, waste signs and supplier identities are unchanged. This reconciles the existing nominal material ledger, not actual plant grades or recycling recovery fractions; no avoided-production credit.</t>
         </is>
       </c>
       <c r="J585"/>

</xml_diff>